<commit_message>
Update main with AISBAFA project files for milestone 3
</commit_message>
<xml_diff>
--- a/Artifacts/Unit_Test_Plan_v0.1.xlsx
+++ b/Artifacts/Unit_Test_Plan_v0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\AIBAFA\Artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD9F53E2-7F27-45E6-9ED6-982CF8DFE50B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9206CECD-7FD7-4E87-9F5B-6BE248E8BFF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C3B83BB6-2AB9-4547-8541-9F6969E92BF1}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="79">
   <si>
     <t>Actual Result</t>
   </si>
@@ -247,13 +247,185 @@
   </si>
   <si>
     <t>Button disabled; prevents redundant calls.</t>
+  </si>
+  <si>
+    <t>Agent4_RootCause_RAG</t>
+  </si>
+  <si>
+    <t>Query Agent 4 with database failure log.</t>
+  </si>
+  <si>
+    <t>Vector store context retrieval &amp; cause hypothesis logic.</t>
+  </si>
+  <si>
+    <t>Cause hypothesis generated with &gt;85% confidence score.</t>
+  </si>
+  <si>
+    <t>Agent5_Code_Patch</t>
+  </si>
+  <si>
+    <t>Pass runtime stack trace to Agent 5.</t>
+  </si>
+  <si>
+    <t>Automated Python code remediation generator.</t>
+  </si>
+  <si>
+    <t>Synthesizes executable code patch with safety guards.</t>
+  </si>
+  <si>
+    <t>Dashboard_5Card_Layout</t>
+  </si>
+  <si>
+    <t>Submit error log on dashboard interface.</t>
+  </si>
+  <si>
+    <t>5-card structured container rendering.</t>
+  </si>
+  <si>
+    <t>Dashboard renders 5 distinct analysis cards cleanly.</t>
+  </si>
+  <si>
+    <t>UI_CodeBlock_Sanitize</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Render remediation code fix containing </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>&amp;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Code patch HTML character escaping in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>&lt;pre&gt;&lt;code&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Patch code displays safely without UI layout breaking.</t>
+  </si>
+  <si>
+    <t>Vector_Match_Clamping</t>
+  </si>
+  <si>
+    <t>Calculate similarity for identical log vectors.</t>
+  </si>
+  <si>
+    <t>Cosine distance evaluation formula and percentage bounding.</t>
+  </si>
+  <si>
+    <t>Returns 100.0% Match score without NaN error.</t>
+  </si>
+  <si>
+    <t>Batch_JSON_Ingestion</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Post </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>.json</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> file containing 50 log items.</t>
+    </r>
+  </si>
+  <si>
+    <t>Asynchronous batch worker queue processing.</t>
+  </si>
+  <si>
+    <t>All 50 log entries processed in &lt;2.5s without locking.</t>
+  </si>
+  <si>
+    <t>Agent_Validation_Suite</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Trigger </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>/api/v1/validate-agents</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> benchmark endpoint.</t>
+    </r>
+  </si>
+  <si>
+    <t>Multi-language error trace fixture evaluation.</t>
+  </si>
+  <si>
+    <t>Benchmark execution completes with &gt;75% accuracy match.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -283,6 +455,11 @@
     <font>
       <sz val="8"/>
       <color rgb="FF1F1F1F"/>
+      <name val="Google Sans Text"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Google Sans Text"/>
       <family val="2"/>
     </font>
@@ -343,7 +520,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -353,6 +530,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -668,7 +851,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF95B16C-182C-4757-B929-A728708A2DB0}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="12.5"/>
   <cols>
     <col min="1" max="1" width="9.1796875" customWidth="1"/>
@@ -926,6 +1109,146 @@
         <v>10</v>
       </c>
     </row>
+    <row r="14" spans="1:6" ht="50.5" thickBot="1">
+      <c r="A14" s="5">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="50.5" thickBot="1">
+      <c r="A15" s="5">
+        <v>13</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="38" thickBot="1">
+      <c r="A16" s="5">
+        <v>14</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="50.5" thickBot="1">
+      <c r="A17" s="5">
+        <v>15</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="50.5" thickBot="1">
+      <c r="A18" s="5">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="38" thickBot="1">
+      <c r="A19" s="5">
+        <v>17</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="63" thickBot="1">
+      <c r="A20" s="5">
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Milestone 4 Updated Code
</commit_message>
<xml_diff>
--- a/Artifacts/Unit_Test_Plan_v0.1.xlsx
+++ b/Artifacts/Unit_Test_Plan_v0.1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\AIBAFA\Artifacts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\AISBAFA\Artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9206CECD-7FD7-4E87-9F5B-6BE248E8BFF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDF59A17-9D27-4D01-9B2B-2BCEC69BA8BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C3B83BB6-2AB9-4547-8541-9F6969E92BF1}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="95">
   <si>
     <t>Actual Result</t>
   </si>
@@ -419,13 +419,119 @@
   </si>
   <si>
     <t>Benchmark execution completes with &gt;75% accuracy match.</t>
+  </si>
+  <si>
+    <t>Analytics_Summary_API</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Query </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>/api/analytics/confidence-summary</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> endpoint.</t>
+    </r>
+  </si>
+  <si>
+    <t>Aggregate confidence score calculation and tier distribution counts.</t>
+  </si>
+  <si>
+    <t>Returns rounded average percentage and correct high/moderate/low volume counts.</t>
+  </si>
+  <si>
+    <t>Analytics_Logs_Filter</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Request </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>/api/analytics/logs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>min_confidence</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> parameter.</t>
+    </r>
+  </si>
+  <si>
+    <t>Optional query string parameter log isolation.</t>
+  </si>
+  <si>
+    <t>Returns filtered execution records matching threshold criteria without errors.</t>
+  </si>
+  <si>
+    <t>Dashboard_Confidence_KPI</t>
+  </si>
+  <si>
+    <t>Render analytics summary header card on dashboard UI.</t>
+  </si>
+  <si>
+    <t>Real-time average confidence percentage display.</t>
+  </si>
+  <si>
+    <t>Header KPI card displays formatted percentage correctly.</t>
+  </si>
+  <si>
+    <t>Confidence_Tier_Badges</t>
+  </si>
+  <si>
+    <t>Populate execution logs table with score values.</t>
+  </si>
+  <si>
+    <t>Dynamic color-coded tier badge rendering (Green, Amber, Rose).</t>
+  </si>
+  <si>
+    <t>Badges apply correct Tailwind CSS styling based on threshold rules.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -534,8 +640,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -851,8 +957,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF95B16C-182C-4757-B929-A728708A2DB0}">
-  <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultRowHeight="12.5"/>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.1796875" customWidth="1"/>
     <col min="2" max="2" width="14.26953125" customWidth="1"/>
@@ -861,7 +967,7 @@
     <col min="6" max="6" width="15.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="31.5" thickBot="1">
+    <row r="1" spans="1:6" ht="31.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
@@ -881,7 +987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="13.5" thickBot="1">
+    <row r="2" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -889,7 +995,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" spans="1:6" ht="38" thickBot="1">
+    <row r="3" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -909,7 +1015,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="38" thickBot="1">
+    <row r="4" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -929,7 +1035,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="38" thickBot="1">
+    <row r="5" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -949,7 +1055,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="38" thickBot="1">
+    <row r="6" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -969,7 +1075,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="38" thickBot="1">
+    <row r="7" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -989,7 +1095,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="38" thickBot="1">
+    <row r="8" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -1009,7 +1115,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="38" thickBot="1">
+    <row r="9" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -1029,7 +1135,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="38" thickBot="1">
+    <row r="10" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -1049,7 +1155,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="38" thickBot="1">
+    <row r="11" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -1069,7 +1175,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="38" thickBot="1">
+    <row r="12" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -1089,7 +1195,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="38" thickBot="1">
+    <row r="13" spans="1:6" ht="38" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -1109,8 +1215,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="50.5" thickBot="1">
-      <c r="A14" s="5">
+    <row r="14" spans="1:6" ht="50.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
         <v>12</v>
       </c>
       <c r="B14" s="4" t="s">
@@ -1129,8 +1235,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="50.5" thickBot="1">
-      <c r="A15" s="5">
+    <row r="15" spans="1:6" ht="50.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="4">
         <v>13</v>
       </c>
       <c r="B15" s="4" t="s">
@@ -1149,8 +1255,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="38" thickBot="1">
-      <c r="A16" s="5">
+    <row r="16" spans="1:6" ht="50.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="4">
         <v>14</v>
       </c>
       <c r="B16" s="4" t="s">
@@ -1169,8 +1275,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="50.5" thickBot="1">
-      <c r="A17" s="5">
+    <row r="17" spans="1:6" ht="63" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="4">
         <v>15</v>
       </c>
       <c r="B17" s="4" t="s">
@@ -1189,8 +1295,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="50.5" thickBot="1">
-      <c r="A18" s="5">
+    <row r="18" spans="1:6" ht="50.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4">
         <v>16</v>
       </c>
       <c r="B18" s="4" t="s">
@@ -1209,8 +1315,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="38" thickBot="1">
-      <c r="A19" s="5">
+    <row r="19" spans="1:6" ht="50.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="4">
         <v>17</v>
       </c>
       <c r="B19" s="4" t="s">
@@ -1229,8 +1335,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="63" thickBot="1">
-      <c r="A20" s="5">
+    <row r="20" spans="1:6" ht="63" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="4">
         <v>18</v>
       </c>
       <c r="B20" s="4" t="s">
@@ -1246,6 +1352,86 @@
         <v>78</v>
       </c>
       <c r="F20" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="75.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
+        <v>19</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="63" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
+        <v>20</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="50.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="2">
+        <v>21</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="50.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>22</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="3" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>